<commit_message>
Audit SACO Phase 2 — troisième passe : contrôles d'identité arithmétique (partie H)
Nouveaux constats vérifiés :
- divergence des tableaux de zone localisée dans la seule colonne d'ajustement
  (identité J = I - moyenne provinciale respectée 64/64 dans les deux fichiers)
- réconciliation exacte des tableaux 11, 12 et 4 (306 CAC, 91 CODESA, 249 unités mobiles)
- 5 CAC hors de la grille de progression déclarée (16,7 / 19,4 / 27,8 points)
- chapitre 8 : 23 séries de quintiles non monotones, 12 IC d'Erreygers sur 24 contenant zéro
Deux griefs retirés (effectifs du tableau 31, écarts de zone).
25 recommandations dont 12 bloquantes ; charge chiffrée 32,5 j-h.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Audit_SACO_Phase2_annexes_2026-10-20.xlsx
+++ b/Audit_SACO_Phase2_annexes_2026-10-20.xlsx
@@ -8,10 +8,11 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Synthèse" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Décisions 78 onglets" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Réconciliation" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommandations" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contrôles identité" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Décisions 78 onglets" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Réconciliation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Figures" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Recommandations" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -433,11 +434,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="90" customWidth="1" min="2" max="2"/>
+    <col width="95" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -460,7 +461,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Seconde passe — 20 octobre 2026</t>
+          <t>Troisième passe — 20 octobre 2026 (parties A à H)</t>
         </is>
       </c>
     </row>
@@ -639,7 +640,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20">
@@ -649,37 +650,47 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Recommandations</t>
+          <t>Griefs retirés après vérification</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>22</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>dont bloquantes</t>
+          <t>Recommandations</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>9</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>dont bloquantes</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Charge chiffrée hors rédaction (j-h)</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>29</v>
+      <c r="B24" t="n">
+        <v>32.5</v>
       </c>
     </row>
   </sheetData>
@@ -688,6 +699,486 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Contrôle</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Périmètre</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Résultat</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Partie</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Évolution = T1 − T0 (zones)</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>4 tableaux × 16 zones</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>15/64 à 0,1 pt</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Écarts d'arrondi d'affichage : les évolutions sont calculées sur les valeurs non arrondies</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Écart = évolution ajustée − moyenne provinciale</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Classeur, 64 cellules</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>64/64</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Identité respectée</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>H.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Écart = évolution ajustée − moyenne provinciale</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Rapport, 64 cellules</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>64/64</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Identité respectée : la divergence est un changement de méthode d'ajustement</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>H.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Évolution ajustée et écart à la moyenne</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Tableaux 21, 22, 54, 55</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>38/128 cellules divergentes</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Concentrées sur P1 (19) et P2 (19) ; P3 et P4 conformes</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>H.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Mouvements = appariement</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Tableau 11 vs tableau 4</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>306 CAC ; 91 CODESA</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Exact ; pourcentages somment à 100</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>H.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Liste nominative = unités mobiles</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>T22 vs T21</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>189 + 60 = 249</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Exact, aucun doublon, delta cohérent 249/249</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>H.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Pas de progression CAC</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>189 unités</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>184 multiples de 11,1</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>5 unités hors grille (16,7 ; 19,4 ; 27,8) — grille réelle 1/36</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>H.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Pas de progression CODESA</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>60 unités</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>60/60 multiples de 14,3</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Conforme</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>H.3</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Monotonie du gradient par quintile</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>32 séries</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>23 non monotones</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Ruptures jusqu'à 20,9 points ; « gradient » impropre</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>H.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>IC des indices d'Erreygers</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>24 indices</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>12 contiennent zéro</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Aucune conclusion possible pour la moitié des indicateurs</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>H.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Sens des évolutions d'inégalité</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>12 séries T0→T1</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>11 diminuent dans les deux bras</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Réduction commune, non attribuable au programme</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>H.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Effectifs du tableau 31</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2 sous-groupes</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>4991 vs 5713</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Bases différentes (analyse vs observations) : grief retiré</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>H.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Écart déclaré − carnet vu</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>20 lignes T44</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>20/20</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Identité respectée</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>G.5</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Colonne n du tableau 60</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>8 lignes</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>8/8</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Exacte au regard du tableau 3</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>G.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Cohérence des IC de l'indice de conformité</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>8 lignes T52</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>2 anomalies</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Largeur d'IC doublée à effectif constant (bras témoin) ; à expliquer</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>H.4</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Libellés de catégories du tableau 9</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>24 lignes</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>2 genres</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>« fonctionnel » / « fonctionnelle » selon l'organe</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>H.6</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3873,7 +4364,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -6591,7 +7082,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -7983,17 +8474,17 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
-    <col width="70" customWidth="1" min="2" max="2"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
@@ -8144,12 +8635,12 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>REC-005</t>
+          <t>REC-016</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Versionnage et horodatage des sorties</t>
+          <t>Exécution du tri des 78 onglets</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -8158,30 +8649,30 @@
         </is>
       </c>
       <c r="D7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="3" t="n">
         <v>1</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>REC-006</t>
+          <t>REC-005</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Recalcul des tableaux dérivés</t>
+          <t>Versionnage et horodatage des sorties</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Bloquant</t>
+          <t>Majeur</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>2</v>
@@ -8190,21 +8681,21 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>REC-020</t>
+          <t>REC-006</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Repondération de second niveau et publication des poids</t>
+          <t>Recalcul des tableaux dérivés</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Majeur</t>
+          <t>Bloquant</t>
         </is>
       </c>
       <c r="D9" s="3" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>2</v>
@@ -8213,21 +8704,21 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>REC-021</t>
+          <t>REC-023</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Règle de calcul de la co-couverture de la cascade</t>
+          <t>Règle d'ajustement des tableaux de zone</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Majeur</t>
+          <t>Bloquant</t>
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>2</v>
@@ -8236,21 +8727,21 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>REC-012</t>
+          <t>REC-020</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Reprise de l'appareil graphique</t>
+          <t>Repondération de second niveau et publication des poids</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Bloquant</t>
+          <t>Majeur</t>
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="E11" s="3" t="n">
         <v>2</v>
@@ -8259,12 +8750,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>REC-013</t>
+          <t>REC-021</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Refonte des fiches de zone</t>
+          <t>Règle de calcul de la co-couverture de la cascade</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -8273,7 +8764,7 @@
         </is>
       </c>
       <c r="D12" s="3" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E12" s="3" t="n">
         <v>2</v>
@@ -8282,21 +8773,21 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>REC-014</t>
+          <t>REC-025</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Scripts, version, journal d'exécution</t>
+          <t>Grille réelle de l'indice de fonctionnalité des CAC</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>Bloquant</t>
+          <t>Majeur</t>
         </is>
       </c>
       <c r="D13" s="3" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E13" s="3" t="n">
         <v>2</v>
@@ -8305,12 +8796,12 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>REC-007</t>
+          <t>REC-012</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Dictionnaire d'indicateurs unique</t>
+          <t>Reprise de l'appareil graphique</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -8322,18 +8813,18 @@
         <v>3</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>REC-008</t>
+          <t>REC-013</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Trois effectifs distingués</t>
+          <t>Refonte des fiches de zone</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -8342,44 +8833,44 @@
         </is>
       </c>
       <c r="D15" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>REC-009</t>
+          <t>REC-014</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Seuils sourcés, grille des cas autoportante</t>
+          <t>Scripts, version, journal d'exécution</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Majeur</t>
+          <t>Bloquant</t>
         </is>
       </c>
       <c r="D16" s="3" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="E16" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>REC-010</t>
+          <t>REC-007</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Identifier le seul primaire conclusif</t>
+          <t>Dictionnaire d'indicateurs unique</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
@@ -8388,7 +8879,7 @@
         </is>
       </c>
       <c r="D17" s="3" t="n">
-        <v>0.5</v>
+        <v>3</v>
       </c>
       <c r="E17" s="3" t="n">
         <v>3</v>
@@ -8397,12 +8888,12 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>REC-011</t>
+          <t>REC-008</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Traiter la variante « sans L6_recent »</t>
+          <t>Trois effectifs distingués</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -8411,7 +8902,7 @@
         </is>
       </c>
       <c r="D18" s="3" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="E18" s="3" t="n">
         <v>3</v>
@@ -8420,12 +8911,12 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>REC-015</t>
+          <t>REC-009</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Contrôles automatiques de diffusion</t>
+          <t>Seuils sourcés, grille des cas autoportante</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -8434,7 +8925,7 @@
         </is>
       </c>
       <c r="D19" s="3" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E19" s="3" t="n">
         <v>3</v>
@@ -8443,44 +8934,44 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>REC-016</t>
+          <t>REC-010</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Exécution du tri des 78 onglets</t>
+          <t>Identifier le seul primaire conclusif</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>Majeur</t>
+          <t>Bloquant</t>
         </is>
       </c>
       <c r="D20" s="3" t="n">
-        <v>2</v>
+        <v>0.5</v>
       </c>
       <c r="E20" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>REC-017</t>
+          <t>REC-011</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>Rédaction du rapport</t>
+          <t>Traiter la variante « sans L6_recent »</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>Bloquant</t>
+          <t>Majeur</t>
         </is>
       </c>
       <c r="D21" s="3" t="n">
-        <v>20</v>
+        <v>0.5</v>
       </c>
       <c r="E21" s="3" t="n">
         <v>3</v>
@@ -8489,12 +8980,12 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>REC-018</t>
+          <t>REC-015</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Revue de validation</t>
+          <t>Contrôles automatiques de diffusion</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -8503,7 +8994,7 @@
         </is>
       </c>
       <c r="D22" s="3" t="n">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="E22" s="3" t="n">
         <v>3</v>
@@ -8512,23 +9003,115 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
+          <t>REC-017</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Rédaction du rapport</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Bloquant</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>REC-018</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Revue de validation</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Majeur</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
           <t>REC-019</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B25" s="3" t="inlineStr">
         <is>
           <t>Déséquilibre initial et effet plafond</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C25" s="3" t="inlineStr">
         <is>
           <t>Majeur</t>
         </is>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D25" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="3" t="n">
+      <c r="E25" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>REC-024</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Nommer le tableau 12 (unités ayant changé)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Majeur</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>REC-026</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Chapitre 8 : ni gradient, ni effet sur l'équité</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Bloquant</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E27" s="3" t="n">
         <v>3</v>
       </c>
     </row>

</xml_diff>